<commit_message>
feat: update template_final.xlsx with new data structure and formatting
</commit_message>
<xml_diff>
--- a/storage/app/private/template/template_final.xlsx
+++ b/storage/app/private/template/template_final.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>kode_kab</t>
   </si>
@@ -158,6 +158,9 @@
   </si>
   <si>
     <t>Kota Batu</t>
+  </si>
+  <si>
+    <t>Provinsi Jawa Timur</t>
   </si>
 </sst>
 </file>
@@ -687,7 +690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="10.1796875" customWidth="1"/>
@@ -1013,6 +1016,14 @@
         <v>41</v>
       </c>
     </row>
+    <row r="40" spans="1:2">
+      <c r="A40">
+        <v>3500</v>
+      </c>
+      <c r="B40" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>